<commit_message>
time normalization valve level made better
</commit_message>
<xml_diff>
--- a/Field-trails/Cattle-Slurry 2025-10-28/soil properties at aplication.xlsx
+++ b/Field-trails/Cattle-Slurry 2025-10-28/soil properties at aplication.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mikae\Desktop\Github - speciale\Larsen-2025-Masterthesis-DFCs\Fall field trails\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mikae\Desktop\Github - speciale\Larsen-2025-Masterthesis-DFCs\Field-trails\Cattle-Slurry 2025-10-28\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ED65D69-9044-4A76-922A-9536CD0F73AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95A15014-3F22-461C-AD6B-0C5735482857}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="360" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -88,8 +88,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -128,11 +129,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -479,7 +481,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09EAA5BB-1777-4A36-A094-C0B46E9D4726}">
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="32.5546875" bestFit="1" customWidth="1"/>
@@ -617,6 +619,16 @@
         <v>0.76457091774482433</v>
       </c>
     </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D8" s="4"/>
+      <c r="F8" s="4"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="F9" s="4"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="F10" s="4"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>